<commit_message>
asset_coverage: Generic and Male/Female anims are mutually exclusive
A class is covered by EITHER a Generic combat anim OR gendered (Male/Female)
ones — not both. So the coverage no longer flags the unneeded route as missing:
- Generic present -> Male/Female shown as "—" (N/A).
- Only gendered present -> Generic shown as "—"; Male/Female show ✅/⬜.
- Nothing present -> Generic ⬜ (make at least that), Male/Female "—".

"—" cells render neutral (white) in the Excel. The summary now counts a class
as covered if it has Generic OR a gender variant.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0173CjjXKMnsNm8AgUP3We9A
</commit_message>
<xml_diff>
--- a/docs/ASSET_COVERAGE.xlsx
+++ b/docs/ASSET_COVERAGE.xlsx
@@ -40,7 +40,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -60,6 +60,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -94,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -108,6 +113,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -513,11 +521,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  con combat anim genérica</t>
+          <t xml:space="preserve">  con combat anim (Generic o género)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6">
@@ -629,7 +637,7 @@
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>Armas anim genérica</t>
+          <t>Armas de la anim</t>
         </is>
       </c>
     </row>
@@ -657,14 +665,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -697,14 +705,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -737,14 +745,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -777,14 +785,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -817,14 +825,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -857,14 +865,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -897,14 +905,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -937,14 +945,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -977,14 +985,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -1017,14 +1025,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -1057,14 +1065,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
@@ -1097,14 +1105,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -1137,14 +1145,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
@@ -1177,14 +1185,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
@@ -1212,9 +1220,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -1229,7 +1237,7 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Javelin, Lance, MagicSword, Sword</t>
         </is>
       </c>
     </row>
@@ -1257,14 +1265,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -1297,14 +1305,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G18" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
@@ -1337,14 +1345,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -1377,14 +1385,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -1417,14 +1425,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -1452,9 +1460,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1469,7 +1477,7 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Axe, HandAxe</t>
         </is>
       </c>
     </row>
@@ -1497,14 +1505,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
@@ -1537,14 +1545,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
@@ -1577,14 +1585,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
@@ -1617,14 +1625,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
@@ -1657,14 +1665,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G27" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
@@ -1697,14 +1705,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G28" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
@@ -1737,14 +1745,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G29" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
@@ -1777,14 +1785,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G30" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
@@ -1817,14 +1825,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G31" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
@@ -1857,14 +1865,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G32" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -1897,14 +1905,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G33" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -1937,14 +1945,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F34" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G34" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
@@ -1977,14 +1985,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F35" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G35" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
@@ -2017,14 +2025,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F36" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G36" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
@@ -2057,14 +2065,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G37" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
@@ -2097,14 +2105,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F38" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G38" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
@@ -2137,14 +2145,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F39" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G39" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
@@ -2177,14 +2185,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G40" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
@@ -2217,14 +2225,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F41" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G41" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
@@ -2257,14 +2265,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F42" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G42" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
@@ -2297,14 +2305,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F43" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G43" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
@@ -2337,14 +2345,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F44" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G44" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
@@ -2377,14 +2385,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F45" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G45" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
@@ -2417,14 +2425,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F46" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G46" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr">
@@ -2457,14 +2465,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F47" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G47" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
@@ -2497,14 +2505,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F48" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G48" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
@@ -2537,14 +2545,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F49" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G49" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
@@ -2577,14 +2585,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F50" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G50" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
@@ -2612,9 +2620,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
@@ -2629,7 +2637,7 @@
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Axe, HandAxe, MagicSword, Sword</t>
         </is>
       </c>
     </row>
@@ -2657,14 +2665,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F52" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G52" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr">
@@ -2697,14 +2705,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F53" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G53" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr">
@@ -2737,14 +2745,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F54" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G54" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H54" s="3" t="inlineStr">
@@ -2772,9 +2780,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
@@ -2789,7 +2797,7 @@
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MagicAnima, MagicStaff, MagicSword, Sword</t>
         </is>
       </c>
     </row>
@@ -2812,9 +2820,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
@@ -2829,7 +2837,7 @@
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MagicAnima, MagicSword, Sword</t>
         </is>
       </c>
     </row>
@@ -2852,9 +2860,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="E57" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
@@ -2869,7 +2877,7 @@
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Axe, Bow, HandAxe, Javelin, Lance, MagicAnima, MagicStaff, MagicSword, Sword</t>
         </is>
       </c>
     </row>
@@ -2897,14 +2905,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F58" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G58" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
@@ -2932,9 +2940,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
@@ -2949,7 +2957,7 @@
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MagicAnima, MagicStaff</t>
         </is>
       </c>
     </row>
@@ -2972,9 +2980,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="E60" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="F60" s="4" t="inlineStr">
@@ -2989,7 +2997,7 @@
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Bow</t>
         </is>
       </c>
     </row>
@@ -3012,9 +3020,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E61" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="E61" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
@@ -3029,7 +3037,7 @@
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MagicSword, Sword</t>
         </is>
       </c>
     </row>
@@ -3057,14 +3065,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F62" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G62" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H62" s="3" t="inlineStr">
@@ -3097,14 +3105,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F63" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G63" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H63" s="3" t="inlineStr">
@@ -3137,14 +3145,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F64" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G64" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G64" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H64" s="3" t="inlineStr">
@@ -3177,14 +3185,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F65" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G65" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F65" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G65" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H65" s="3" t="inlineStr">
@@ -3217,14 +3225,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F66" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G66" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F66" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G66" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H66" s="3" t="inlineStr">
@@ -3257,14 +3265,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F67" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="G67" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F67" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G67" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H67" s="3" t="inlineStr">
@@ -3545,7 +3553,7 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>⚠️</t>
         </is>
@@ -3767,7 +3775,7 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>⚠️</t>
         </is>
@@ -4988,7 +4996,7 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F46" s="6" t="inlineStr">
+      <c r="F46" s="7" t="inlineStr">
         <is>
           <t>⚠️</t>
         </is>
@@ -5099,7 +5107,7 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F49" s="6" t="inlineStr">
+      <c r="F49" s="7" t="inlineStr">
         <is>
           <t>⚠️</t>
         </is>
@@ -5321,7 +5329,7 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F55" s="6" t="inlineStr">
+      <c r="F55" s="7" t="inlineStr">
         <is>
           <t>⚠️</t>
         </is>
@@ -5358,7 +5366,7 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F56" s="6" t="inlineStr">
+      <c r="F56" s="7" t="inlineStr">
         <is>
           <t>⚠️</t>
         </is>
@@ -5395,7 +5403,7 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F57" s="6" t="inlineStr">
+      <c r="F57" s="7" t="inlineStr">
         <is>
           <t>⚠️</t>
         </is>
@@ -5722,12 +5730,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>Problema</t>
         </is>

</xml_diff>

<commit_message>
Rename classes/units/portraits for canonical naming
- PreHero class -> Mercenary (id/map_sprite_nid/combat_anim_nid), keep the
  in-game display name Swordfighter; reassign Holyn/FakeHolyn.
- Merge AThief + BThief + BThief_Lara into a single Thief class; reassign
  Dew/Lifis (thieves) and Lara.
- Rename the paladin triplets guarding Lachesis: Alva->Alvar, Eva->Evan,
  Eve->Evar (units, level 2 deploys, events, portrait offsets, portrait
  assets).
- Rename portraits AlvaFE4->Alvar and AlvaFE5->Alva.
- Regenerate docs/ASSET_COVERAGE.{md,xlsx} to reflect the renames.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0173CjjXKMnsNm8AgUP3We9A
</commit_message>
<xml_diff>
--- a/docs/ASSET_COVERAGE.xlsx
+++ b/docs/ASSET_COVERAGE.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Problemas" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Clases'!$A$1:$H$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Clases'!$A$1:$H$65</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Personajes'!$A$1:$G$65</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4">
@@ -515,7 +515,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5">
@@ -586,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -844,7 +844,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>AThief</t>
+          <t>Archer</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
@@ -877,14 +877,14 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>MagicSword, Sword</t>
+          <t>Bow</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Archer</t>
+          <t>Armour</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
@@ -917,14 +917,14 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Bow</t>
+          <t>Axe, Bow, HandAxe, Javelin, Lance, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Armour</t>
+          <t>Ballistae</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
@@ -940,9 +940,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -957,14 +957,14 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Axe, Bow, HandAxe, Javelin, Lance, MagicSword, Sword</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>BThief</t>
+          <t>Bandit</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
@@ -980,9 +980,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -997,14 +997,14 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Axe, HandAxe</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>BThief_Lara</t>
+          <t>Barbarian</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
@@ -1020,9 +1020,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -1037,14 +1037,14 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Axe, HandAxe</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Ballistae</t>
+          <t>Bard</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
@@ -1084,7 +1084,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Bandit</t>
+          <t>Cavalier</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
@@ -1100,31 +1100,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Axe, HandAxe</t>
+          <t>Javelin, Lance, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Barbarian</t>
+          <t>CavalierA</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
@@ -1164,7 +1164,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Bard</t>
+          <t>CavalierB</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
@@ -1204,7 +1204,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Cavalier</t>
+          <t>CavalierL</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
@@ -1220,31 +1220,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>Javelin, Lance, MagicSword, Sword</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>CavalierA</t>
+          <t>CavalierS</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
@@ -1260,9 +1260,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -1277,14 +1277,14 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Axe, HandAxe</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>CavalierB</t>
+          <t>DragonKnight</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
@@ -1300,9 +1300,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -1317,14 +1317,14 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Javelin, Lance, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>CavalierL</t>
+          <t>Fighter</t>
         </is>
       </c>
       <c r="B19" s="3" t="n">
@@ -1340,31 +1340,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Axe, HandAxe</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>CavalierS</t>
+          <t>LightPriestess</t>
         </is>
       </c>
       <c r="B20" s="3" t="n">
@@ -1404,7 +1404,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>DragonKnight</t>
+          <t>LoptoMage</t>
         </is>
       </c>
       <c r="B21" s="3" t="n">
@@ -1420,9 +1420,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -1437,14 +1437,14 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Javelin, Lance, MagicSword, Sword</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Fighter</t>
+          <t>LordLeaf</t>
         </is>
       </c>
       <c r="B22" s="3" t="n">
@@ -1460,31 +1460,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>Axe, HandAxe</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>LightPriestess</t>
+          <t>LordSeliph</t>
         </is>
       </c>
       <c r="B23" s="3" t="n">
@@ -1524,7 +1524,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>LoptoMage</t>
+          <t>Mage</t>
         </is>
       </c>
       <c r="B24" s="3" t="n">
@@ -1564,7 +1564,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>LordLeaf</t>
+          <t>Mercenary</t>
         </is>
       </c>
       <c r="B25" s="3" t="n">
@@ -1604,7 +1604,7 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>LordSeliph</t>
+          <t>PegasusKnight</t>
         </is>
       </c>
       <c r="B26" s="3" t="n">
@@ -1644,7 +1644,7 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Mage</t>
+          <t>Pirate</t>
         </is>
       </c>
       <c r="B27" s="3" t="n">
@@ -1660,9 +1660,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
@@ -1677,14 +1677,14 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Axe, HandAxe, MagicStaff</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>PegasusKnight</t>
+          <t>Priest</t>
         </is>
       </c>
       <c r="B28" s="3" t="n">
@@ -1700,9 +1700,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
@@ -1717,14 +1717,14 @@
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MagicStaff</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Pirate</t>
+          <t>Priestess</t>
         </is>
       </c>
       <c r="B29" s="3" t="n">
@@ -1757,14 +1757,14 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>Axe, HandAxe, MagicStaff</t>
+          <t>MagicStaff</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>PreHero</t>
+          <t>Princess</t>
         </is>
       </c>
       <c r="B30" s="3" t="n">
@@ -1804,7 +1804,7 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Priest</t>
+          <t>Soldier</t>
         </is>
       </c>
       <c r="B31" s="3" t="n">
@@ -1837,14 +1837,14 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>MagicStaff</t>
+          <t>Javelin, Lance</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Priestess</t>
+          <t>Swordfighter</t>
         </is>
       </c>
       <c r="B32" s="3" t="n">
@@ -1860,9 +1860,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
@@ -1877,14 +1877,14 @@
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>MagicStaff</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Princess</t>
+          <t>Thief</t>
         </is>
       </c>
       <c r="B33" s="3" t="n">
@@ -1900,9 +1900,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
@@ -1917,14 +1917,14 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Soldier</t>
+          <t>Troubadour</t>
         </is>
       </c>
       <c r="B34" s="3" t="n">
@@ -1957,18 +1957,18 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>Javelin, Lance</t>
+          <t>MagicStaff, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Swordfighter</t>
+          <t>APaladin</t>
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
@@ -2004,11 +2004,11 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Troubadour</t>
+          <t>BPaladin</t>
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
@@ -2020,9 +2020,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
@@ -2037,14 +2037,14 @@
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>MagicStaff, MagicSword, Sword</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>APaladin</t>
+          <t>Berserker</t>
         </is>
       </c>
       <c r="B37" s="3" t="n">
@@ -2060,9 +2060,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
@@ -2077,14 +2077,14 @@
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Axe, HandAxe</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>BPaladin</t>
+          <t>Bishop</t>
         </is>
       </c>
       <c r="B38" s="3" t="n">
@@ -2100,9 +2100,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
@@ -2117,14 +2117,14 @@
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MagicAnima, MagicStaff</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Berserker</t>
+          <t>BowKnight</t>
         </is>
       </c>
       <c r="B39" s="3" t="n">
@@ -2157,14 +2157,14 @@
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>Axe, HandAxe</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Bishop</t>
+          <t>Dancer</t>
         </is>
       </c>
       <c r="B40" s="3" t="n">
@@ -2197,14 +2197,14 @@
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima, MagicStaff</t>
+          <t>MagicSword, Refresh, Sword</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>BowKnight</t>
+          <t>Dancer_Lara</t>
         </is>
       </c>
       <c r="B41" s="3" t="n">
@@ -2237,14 +2237,14 @@
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MagicSword, Refresh, Sword</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Dancer</t>
+          <t>DarkSage</t>
         </is>
       </c>
       <c r="B42" s="3" t="n">
@@ -2260,9 +2260,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
@@ -2277,14 +2277,14 @@
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>MagicSword, Refresh, Sword</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Dancer_Lara</t>
+          <t>DragonMaster</t>
         </is>
       </c>
       <c r="B43" s="3" t="n">
@@ -2317,14 +2317,14 @@
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>MagicSword, Refresh, Sword</t>
+          <t>Javelin, Lance, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>DarkSage</t>
+          <t>DukeKnight</t>
         </is>
       </c>
       <c r="B44" s="3" t="n">
@@ -2364,7 +2364,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>DragonMaster</t>
+          <t>FalconKnight</t>
         </is>
       </c>
       <c r="B45" s="3" t="n">
@@ -2404,7 +2404,7 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>DukeKnight</t>
+          <t>ForrestKnight</t>
         </is>
       </c>
       <c r="B46" s="3" t="n">
@@ -2444,7 +2444,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>FalconKnight</t>
+          <t>General</t>
         </is>
       </c>
       <c r="B47" s="3" t="n">
@@ -2477,14 +2477,14 @@
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>Javelin, Lance, MagicSword, Sword</t>
+          <t>Axe, Bow, HandAxe, Javelin, Lance, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>ForrestKnight</t>
+          <t>GreatKnight</t>
         </is>
       </c>
       <c r="B48" s="3" t="n">
@@ -2524,7 +2524,7 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="B49" s="3" t="n">
@@ -2540,31 +2540,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E49" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G49" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>Axe, Bow, HandAxe, Javelin, Lance, MagicSword, Sword</t>
+          <t>Axe, HandAxe, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>GreatKnight</t>
+          <t>HighPriest</t>
         </is>
       </c>
       <c r="B50" s="3" t="n">
@@ -2604,7 +2604,7 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>HighPriestess</t>
         </is>
       </c>
       <c r="B51" s="3" t="n">
@@ -2620,31 +2620,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E51" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F51" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G51" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>Axe, HandAxe, MagicSword, Sword</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>HighPriest</t>
+          <t>LordKnight</t>
         </is>
       </c>
       <c r="B52" s="3" t="n">
@@ -2684,7 +2684,7 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>HighPriestess</t>
+          <t>MageFighter</t>
         </is>
       </c>
       <c r="B53" s="3" t="n">
@@ -2700,31 +2700,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G53" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="E53" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MagicAnima, MagicStaff, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>LordKnight</t>
+          <t>MageKnight</t>
         </is>
       </c>
       <c r="B54" s="3" t="n">
@@ -2740,31 +2740,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G54" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MagicAnima, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>MageFighter</t>
+          <t>MasterKnight</t>
         </is>
       </c>
       <c r="B55" s="3" t="n">
@@ -2797,14 +2797,14 @@
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima, MagicStaff, MagicSword, Sword</t>
+          <t>Axe, Bow, HandAxe, Javelin, Lance, MagicAnima, MagicStaff, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>MageKnight</t>
+          <t>Rogue</t>
         </is>
       </c>
       <c r="B56" s="3" t="n">
@@ -2820,31 +2820,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E56" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F56" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G56" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima, MagicSword, Sword</t>
+          <t>MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>MasterKnight</t>
+          <t>Sage</t>
         </is>
       </c>
       <c r="B57" s="3" t="n">
@@ -2877,14 +2877,14 @@
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>Axe, Bow, HandAxe, Javelin, Lance, MagicAnima, MagicStaff, MagicSword, Sword</t>
+          <t>MagicAnima, MagicStaff</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Rogue</t>
+          <t>Sniper</t>
         </is>
       </c>
       <c r="B58" s="3" t="n">
@@ -2900,31 +2900,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E58" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F58" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G58" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>MagicSword, Sword</t>
+          <t>Bow</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>Sage</t>
+          <t>Swordmaster</t>
         </is>
       </c>
       <c r="B59" s="3" t="n">
@@ -2957,14 +2957,14 @@
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima, MagicStaff</t>
+          <t>MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>Sniper</t>
+          <t>Warrior</t>
         </is>
       </c>
       <c r="B60" s="3" t="n">
@@ -2980,35 +2980,35 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E60" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F60" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G60" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>Bow</t>
+          <t>Axe, Bow, HandAxe</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Swordmaster</t>
+          <t>Baron</t>
         </is>
       </c>
       <c r="B61" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
@@ -3020,35 +3020,35 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E61" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F61" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G61" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G61" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>MagicSword, Sword</t>
+          <t>Axe, Bow, HandAxe, Javelin, Lance, MagicAnima, MagicStaff, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>Warrior</t>
+          <t>DarkBishop</t>
         </is>
       </c>
       <c r="B62" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
@@ -3077,14 +3077,14 @@
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>Axe, Bow, HandAxe</t>
+          <t>MagicAnima, MagicStaff</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Baron</t>
+          <t>DarkPrince</t>
         </is>
       </c>
       <c r="B63" s="3" t="n">
@@ -3117,14 +3117,14 @@
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>Axe, Bow, HandAxe, Javelin, Lance, MagicAnima, MagicStaff, MagicSword, Sword</t>
+          <t>MagicAnima, MagicStaff</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>DarkBishop</t>
+          <t>Emperor</t>
         </is>
       </c>
       <c r="B64" s="3" t="n">
@@ -3157,14 +3157,14 @@
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima, MagicStaff</t>
+          <t>Axe, Bow, HandAxe, Javelin, Lance, MagicAnima, MagicStaff, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>DarkPrince</t>
+          <t>Queen</t>
         </is>
       </c>
       <c r="B65" s="3" t="n">
@@ -3180,9 +3180,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E65" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="F65" s="6" t="inlineStr">
@@ -3197,92 +3197,12 @@
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima, MagicStaff</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="3" t="inlineStr">
-        <is>
-          <t>Emperor</t>
-        </is>
-      </c>
-      <c r="B66" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="C66" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D66" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E66" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F66" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G66" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H66" s="3" t="inlineStr">
-        <is>
-          <t>Axe, Bow, HandAxe, Javelin, Lance, MagicAnima, MagicStaff, MagicSword, Sword</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="3" t="inlineStr">
-        <is>
-          <t>Queen</t>
-        </is>
-      </c>
-      <c r="B67" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="C67" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D67" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E67" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="F67" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G67" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H67" s="3" t="inlineStr">
-        <is>
           <t>—</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H67"/>
+  <autoFilter ref="A1:H65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3345,7 +3265,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>AlvaFE4</t>
+          <t>Alvar</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -3419,7 +3339,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Eva</t>
+          <t>Evan</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -3456,7 +3376,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Eve</t>
+          <t>Evar</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -3493,12 +3413,12 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Dew</t>
+          <t>Jamke</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>AThief</t>
+          <t>Archer</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -3523,19 +3443,19 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>MagicSword, Sword</t>
+          <t>Bow</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Lifis</t>
+          <t>Ronan</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>AThief</t>
+          <t>Archer</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -3553,21 +3473,21 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>⚠️</t>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>MagicSword, Sword</t>
+          <t>Bow</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Jamke</t>
+          <t>Tanya</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -3577,7 +3497,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -3604,12 +3524,12 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Ronan</t>
+          <t>Arden</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Archer</t>
+          <t>Armour</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -3627,31 +3547,31 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Bow</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Tanya</t>
+          <t>Weissman</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Archer</t>
+          <t>Armour</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -3664,26 +3584,26 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Bow</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Arden</t>
+          <t>Marty</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Armour</t>
+          <t>Bandit</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -3715,12 +3635,12 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Weissman</t>
+          <t>Lewyn</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Armour</t>
+          <t>Bard</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -3728,9 +3648,9 @@
           <t>M</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -3752,17 +3672,17 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Lara</t>
+          <t>Chagall</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>BThief_Lara</t>
+          <t>Baron</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -3775,26 +3695,26 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>⚠️</t>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>MagicSword, Sword</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Marty</t>
+          <t>Raydrik</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Bandit</t>
+          <t>Baron</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -3826,12 +3746,12 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Lewyn</t>
+          <t>Clement</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Bard</t>
+          <t>Bishop</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -3839,9 +3759,9 @@
           <t>M</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -3863,12 +3783,12 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Chagall</t>
+          <t>Alec</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Baron</t>
+          <t>Cavalier</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -3900,12 +3820,12 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Raydrik</t>
+          <t>Noish</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Baron</t>
+          <t>Cavalier</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -3937,12 +3857,12 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Clement</t>
+          <t>NordionGuard</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Bishop</t>
+          <t>Cavalier</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -3950,9 +3870,9 @@
           <t>M</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -3974,12 +3894,12 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Alec</t>
+          <t>Lex</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Cavalier</t>
+          <t>CavalierA</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -3997,26 +3917,26 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Axe, HandAxe</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Noish</t>
+          <t>Midir</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Cavalier</t>
+          <t>CavalierB</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -4048,12 +3968,12 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>NordionGuard</t>
+          <t>Finn</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Cavalier</t>
+          <t>CavalierL</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -4085,12 +4005,12 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Lex</t>
+          <t>Beowulf</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>CavalierA</t>
+          <t>CavalierS</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -4108,26 +4028,26 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Axe, HandAxe</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Midir</t>
+          <t>Coirpre</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>CavalierB</t>
+          <t>Child</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -4159,12 +4079,12 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Finn</t>
+          <t>Sylvia</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>CavalierL</t>
+          <t>Dancer</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -4172,9 +4092,9 @@
           <t>M</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -4196,12 +4116,12 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Beowulf</t>
+          <t>Sandima</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>CavalierS</t>
+          <t>DarkSage</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -4233,12 +4153,12 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Coirpre</t>
+          <t>Elliot</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Child</t>
+          <t>DukeKnight</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -4270,12 +4190,12 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Sylvia</t>
+          <t>Quan</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Dancer</t>
+          <t>DukeKnight</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -4307,12 +4227,12 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Sandima</t>
+          <t>Zain</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>DarkSage</t>
+          <t>DukeKnight</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -4344,12 +4264,12 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Elliot</t>
+          <t>DiMaggio</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>DukeKnight</t>
+          <t>Fighter</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -4367,26 +4287,26 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Axe, HandAxe</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Quan</t>
+          <t>Gerrard</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>DukeKnight</t>
+          <t>Fighter</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -4404,26 +4324,26 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Axe, HandAxe</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Zain</t>
+          <t>Halvan</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>DukeKnight</t>
+          <t>Fighter</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -4441,21 +4361,21 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Axe, HandAxe</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>DiMaggio</t>
+          <t>Osian</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -4492,12 +4412,12 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Gerrard</t>
+          <t>Voltz</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Fighter</t>
+          <t>ForrestKnight</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -4515,26 +4435,26 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Axe, HandAxe</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Halvan</t>
+          <t>Boldor</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Fighter</t>
+          <t>General</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -4552,26 +4472,26 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Axe, HandAxe</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Osian</t>
+          <t>Lobos</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Fighter</t>
+          <t>General</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -4589,26 +4509,26 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Axe, HandAxe</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Voltz</t>
+          <t>Macbeth</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>ForrestKnight</t>
+          <t>General</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -4640,7 +4560,7 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Boldor</t>
+          <t>Phillip</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -4677,12 +4597,12 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Lobos</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>HighPriest</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -4714,17 +4634,17 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Macbeth</t>
+          <t>Deirdre</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>LightPriestess</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -4751,12 +4671,12 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Phillip</t>
+          <t>Sigurd</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>LordKnight</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -4774,26 +4694,26 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Javelin, Lance, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Leif</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>HighPriest</t>
+          <t>LordLeaf</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -4811,31 +4731,31 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F41" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Deirdre</t>
+          <t>Azel</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>LightPriestess</t>
+          <t>Mage</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -4862,12 +4782,12 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Sigurd</t>
+          <t>Tailtiu</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>LordKnight</t>
+          <t>Mage</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -4885,26 +4805,26 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F43" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>⚠️</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>Javelin, Lance, MagicSword, Sword</t>
+          <t>MagicAnima, MagicStaff, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Leif</t>
+          <t>FakeHolyn</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>LordLeaf</t>
+          <t>Mercenary</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -4922,26 +4842,26 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>MagicSword, Sword</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Azel</t>
+          <t>Holyn</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Mage</t>
+          <t>Mercenary</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -4959,26 +4879,26 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F45" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>⚠️</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Axe, HandAxe, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>Tailtiu</t>
+          <t>Erinys</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Mage</t>
+          <t>PegasusKnight</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -4996,31 +4916,31 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F46" s="7" t="inlineStr">
-        <is>
-          <t>⚠️</t>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima, MagicStaff, MagicSword, Sword</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Erinys</t>
+          <t>Aideen</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>PegasusKnight</t>
+          <t>Priestess</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -5047,17 +4967,17 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>FakeHolyn</t>
+          <t>Safy</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>PreHero</t>
+          <t>Priestess</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -5070,31 +4990,31 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F48" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MagicStaff</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Holyn</t>
+          <t>Lachesis</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>PreHero</t>
+          <t>Princess</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -5107,36 +5027,36 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F49" s="7" t="inlineStr">
-        <is>
-          <t>⚠️</t>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>Axe, HandAxe, MagicSword, Sword</t>
+          <t>MagicStaff, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>Aideen</t>
+          <t>Arvis</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Priestess</t>
+          <t>Sage</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -5144,26 +5064,26 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F50" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MagicAnima, MagicStaff</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>Safy</t>
+          <t>Brigid</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Priestess</t>
+          <t>Sniper</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -5181,26 +5101,26 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F51" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>MagicStaff</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>Lachesis</t>
+          <t>Ayra</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Princess</t>
+          <t>Swordfighter</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -5218,36 +5138,36 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F52" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>⚠️</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>MagicStaff, MagicSword, Sword</t>
+          <t>MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>Arvis</t>
+          <t>Mareeta</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Sage</t>
+          <t>Swordfighter</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -5255,31 +5175,31 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F53" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="F53" s="7" t="inlineStr">
+        <is>
+          <t>⚠️</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima, MagicStaff</t>
+          <t>MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>Brigid</t>
+          <t>Shiva</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Sniper</t>
+          <t>Swordfighter</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -5292,26 +5212,26 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F54" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>⚠️</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Ayra</t>
+          <t>Eyvel</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Swordfighter</t>
+          <t>Swordmaster</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -5329,9 +5249,9 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F55" s="7" t="inlineStr">
-        <is>
-          <t>⚠️</t>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
@@ -5343,17 +5263,17 @@
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Mareeta</t>
+          <t>Dew</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Swordfighter</t>
+          <t>Thief</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -5366,9 +5286,9 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F56" s="7" t="inlineStr">
-        <is>
-          <t>⚠️</t>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="G56" s="3" t="inlineStr">
@@ -5380,17 +5300,17 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Shiva</t>
+          <t>Lara</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Swordfighter</t>
+          <t>Thief</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -5417,17 +5337,17 @@
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Eyvel</t>
+          <t>Lifis</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Swordmaster</t>
+          <t>Thief</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
@@ -5440,9 +5360,9 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F58" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>⚠️</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
@@ -5757,7 +5677,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>'Holyn' (PreHero): anim en Hero_Holyn/ pero combat_anim_nid="PreHero" -&gt; el resolver busca PreHero_Holyn (no existe). Renombrar la carpeta a PreHero_Holyn o corregir combat_anim_nid.</t>
+          <t>'Holyn' (Mercenary): anim en Hero_Holyn/ pero combat_anim_nid="Mercenary" -&gt; el resolver busca Mercenary_Holyn (no existe). Renombrar la carpeta a Mercenary_Holyn o corregir combat_anim_nid.</t>
         </is>
       </c>
     </row>
@@ -5777,7 +5697,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>'Lara' (BThief_Lara): anim en Rogue_Lara/ pero combat_anim_nid="ThiefFemale" -&gt; el resolver busca ThiefFemale_Lara (no existe). Renombrar la carpeta a ThiefFemale_Lara o corregir combat_anim_nid.</t>
+          <t>'Lara' (Thief): anim en Rogue_Lara/ pero combat_anim_nid="Thief" -&gt; el resolver busca Thief_Lara (no existe). Renombrar la carpeta a Thief_Lara o corregir combat_anim_nid.</t>
         </is>
       </c>
     </row>
@@ -5787,7 +5707,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>'Lifis' (AThief): anim en Rogue_Lifis/ pero combat_anim_nid="Thief" -&gt; el resolver busca Thief_Lifis (no existe). Renombrar la carpeta a Thief_Lifis o corregir combat_anim_nid.</t>
+          <t>'Lifis' (Thief): anim en Rogue_Lifis/ pero combat_anim_nid="Thief" -&gt; el resolver busca Thief_Lifis (no existe). Renombrar la carpeta a Thief_Lifis o corregir combat_anim_nid.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Unify Dancer_Lara into Dancer; remove Child class; exclude Tester from audit
- Delete Dancer_Lara class: LaraPromotion.gd already keys Lara's special
  dancer behaviour (Dancer<->Rogue re-promotion, shared level) on nid=='Lara'
  and uses the plain 'Dancer' class, so the separate class was already unused.
  Lara can do things other dancers can't purely via that character check.
- Remove the Child class and reassign Coirpre to Priest (his FE5 healer
  class); Coirpre now resolves both a map sprite and a combat anim.
- resource_audit.py: treat Tester as a debug class (tests other units' assets)
  and exclude it from the missing-resource report.

classes.json 63 -> 61. No dangling klass/promotion references. Coverage/audit
docs regenerated.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0173CjjXKMnsNm8AgUP3We9A
</commit_message>
<xml_diff>
--- a/docs/ASSET_COVERAGE.xlsx
+++ b/docs/ASSET_COVERAGE.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Problemas" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Clases'!$A$1:$H$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Clases'!$A$1:$H$62</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Personajes'!$A$1:$G$123</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4">
@@ -515,7 +515,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5">
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6">
@@ -586,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -644,7 +644,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Child</t>
+          <t>Citizen</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
@@ -684,7 +684,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Citizen</t>
+          <t>DragonRider</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
@@ -700,9 +700,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -717,14 +717,14 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Javelin, Lance, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>DragonRider</t>
+          <t>PegasusRider</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
@@ -764,7 +764,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>PegasusRider</t>
+          <t>Tester</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
@@ -780,9 +780,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -797,18 +797,18 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Javelin, Lance, MagicSword, Sword</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Tester</t>
+          <t>Archer</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
@@ -820,9 +820,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -837,14 +837,14 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Bow</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Archer</t>
+          <t>Armour</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
@@ -877,14 +877,14 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Bow</t>
+          <t>Axe, Bow, HandAxe, Javelin, Lance, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Armour</t>
+          <t>Ballistae</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
@@ -900,9 +900,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -917,14 +917,14 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Axe, Bow, HandAxe, Javelin, Lance, MagicSword, Sword</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Ballistae</t>
+          <t>Bandit</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
@@ -940,9 +940,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -957,14 +957,14 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Axe, HandAxe</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Bandit</t>
+          <t>Barbarian</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
@@ -1004,7 +1004,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Barbarian</t>
+          <t>Bard</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
@@ -1020,9 +1020,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -1037,14 +1037,14 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Axe, HandAxe</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Bard</t>
+          <t>Cavalier</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
@@ -1060,31 +1060,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Javelin, Lance, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Cavalier</t>
+          <t>CavalierA</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
@@ -1100,31 +1100,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Javelin, Lance, MagicSword, Sword</t>
+          <t>Axe, HandAxe</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>CavalierA</t>
+          <t>CavalierB</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
@@ -1140,31 +1140,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>Axe, HandAxe</t>
+          <t>Bow</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>CavalierB</t>
+          <t>CavalierL</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
@@ -1180,31 +1180,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Bow</t>
+          <t>Javelin, Lance</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>CavalierL</t>
+          <t>CavalierS</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
@@ -1237,14 +1237,14 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>Javelin, Lance</t>
+          <t>MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>CavalierS</t>
+          <t>DragonKnight</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
@@ -1277,14 +1277,14 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>MagicSword, Sword</t>
+          <t>Javelin, Lance, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>DragonKnight</t>
+          <t>Fighter</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
@@ -1300,31 +1300,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>Javelin, Lance, MagicSword, Sword</t>
+          <t>Axe, HandAxe</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Fighter</t>
+          <t>LightPriestess</t>
         </is>
       </c>
       <c r="B19" s="3" t="n">
@@ -1340,31 +1340,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Axe, HandAxe</t>
+          <t>MagicAnima, MagicStaff</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>LightPriestess</t>
+          <t>LoptoMage</t>
         </is>
       </c>
       <c r="B20" s="3" t="n">
@@ -1404,7 +1404,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>LoptoMage</t>
+          <t>LordLeaf</t>
         </is>
       </c>
       <c r="B21" s="3" t="n">
@@ -1420,9 +1420,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -1437,14 +1437,14 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima, MagicStaff</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>LordLeaf</t>
+          <t>LordSeliph</t>
         </is>
       </c>
       <c r="B22" s="3" t="n">
@@ -1484,7 +1484,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>LordSeliph</t>
+          <t>Mage</t>
         </is>
       </c>
       <c r="B23" s="3" t="n">
@@ -1524,7 +1524,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Mage</t>
+          <t>Mercenary</t>
         </is>
       </c>
       <c r="B24" s="3" t="n">
@@ -1540,31 +1540,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Axe, HandAxe, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Mercenary</t>
+          <t>PegasusKnight</t>
         </is>
       </c>
       <c r="B25" s="3" t="n">
@@ -1580,31 +1580,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>Axe, HandAxe, MagicSword, Sword</t>
+          <t>Javelin, Lance, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>PegasusKnight</t>
+          <t>Pirate</t>
         </is>
       </c>
       <c r="B26" s="3" t="n">
@@ -1637,14 +1637,14 @@
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>Javelin, Lance, MagicSword, Sword</t>
+          <t>Axe, HandAxe, MagicStaff</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Pirate</t>
+          <t>Priest</t>
         </is>
       </c>
       <c r="B27" s="3" t="n">
@@ -1677,14 +1677,14 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>Axe, HandAxe, MagicStaff</t>
+          <t>MagicStaff</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Priest</t>
+          <t>Priestess</t>
         </is>
       </c>
       <c r="B28" s="3" t="n">
@@ -1724,7 +1724,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Priestess</t>
+          <t>Princess</t>
         </is>
       </c>
       <c r="B29" s="3" t="n">
@@ -1740,9 +1740,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
@@ -1757,14 +1757,14 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>MagicStaff</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Princess</t>
+          <t>Soldier</t>
         </is>
       </c>
       <c r="B30" s="3" t="n">
@@ -1780,9 +1780,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
@@ -1797,14 +1797,14 @@
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Javelin, Lance</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Soldier</t>
+          <t>Swordfighter</t>
         </is>
       </c>
       <c r="B31" s="3" t="n">
@@ -1820,31 +1820,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>Javelin, Lance</t>
+          <t>MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Swordfighter</t>
+          <t>Thief</t>
         </is>
       </c>
       <c r="B32" s="3" t="n">
@@ -1860,19 +1860,19 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E32" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -1884,7 +1884,7 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Thief</t>
+          <t>Troubadour</t>
         </is>
       </c>
       <c r="B33" s="3" t="n">
@@ -1917,18 +1917,18 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>MagicSword, Sword</t>
+          <t>MagicStaff, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Troubadour</t>
+          <t>Berserker</t>
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
@@ -1957,14 +1957,14 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>MagicStaff, MagicSword, Sword</t>
+          <t>Axe, HandAxe</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Berserker</t>
+          <t>Bishop</t>
         </is>
       </c>
       <c r="B35" s="3" t="n">
@@ -1997,14 +1997,14 @@
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>Axe, HandAxe</t>
+          <t>MagicAnima, MagicStaff</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Bishop</t>
+          <t>BowKnight</t>
         </is>
       </c>
       <c r="B36" s="3" t="n">
@@ -2037,14 +2037,14 @@
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima, MagicStaff</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>BowKnight</t>
+          <t>Dancer</t>
         </is>
       </c>
       <c r="B37" s="3" t="n">
@@ -2077,14 +2077,14 @@
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MagicSword, Refresh, Sword</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Dancer</t>
+          <t>DarkMage</t>
         </is>
       </c>
       <c r="B38" s="3" t="n">
@@ -2117,14 +2117,14 @@
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>MagicSword, Refresh, Sword</t>
+          <t>MagicAnima</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Dancer_Lara</t>
+          <t>DragonMaster</t>
         </is>
       </c>
       <c r="B39" s="3" t="n">
@@ -2157,14 +2157,14 @@
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>MagicSword, Refresh, Sword</t>
+          <t>Javelin, Lance, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>DarkMage</t>
+          <t>DukeKnight</t>
         </is>
       </c>
       <c r="B40" s="3" t="n">
@@ -2180,9 +2180,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
@@ -2197,14 +2197,14 @@
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>DragonMaster</t>
+          <t>FalconKnight</t>
         </is>
       </c>
       <c r="B41" s="3" t="n">
@@ -2244,7 +2244,7 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>DukeKnight</t>
+          <t>ForrestKnight</t>
         </is>
       </c>
       <c r="B42" s="3" t="n">
@@ -2284,7 +2284,7 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>FalconKnight</t>
+          <t>General</t>
         </is>
       </c>
       <c r="B43" s="3" t="n">
@@ -2317,14 +2317,14 @@
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>Javelin, Lance, MagicSword, Sword</t>
+          <t>Axe, Bow, HandAxe, Javelin, Lance, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>ForrestKnight</t>
+          <t>GreatKnight</t>
         </is>
       </c>
       <c r="B44" s="3" t="n">
@@ -2364,7 +2364,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="B45" s="3" t="n">
@@ -2380,31 +2380,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G45" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>Axe, Bow, HandAxe, Javelin, Lance, MagicSword, Sword</t>
+          <t>Axe, HandAxe, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>GreatKnight</t>
+          <t>HighPriest</t>
         </is>
       </c>
       <c r="B46" s="3" t="n">
@@ -2420,9 +2420,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
@@ -2437,14 +2437,14 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MagicAnima, MagicStaff</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>HighPriestess</t>
         </is>
       </c>
       <c r="B47" s="3" t="n">
@@ -2460,31 +2460,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E47" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G47" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>Axe, HandAxe, MagicSword, Sword</t>
+          <t>MagicAnima, MagicStaff</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>HighPriest</t>
+          <t>LordKnight</t>
         </is>
       </c>
       <c r="B48" s="3" t="n">
@@ -2500,9 +2500,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
@@ -2517,14 +2517,14 @@
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima, MagicStaff</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>HighPriestess</t>
+          <t>MageFighter</t>
         </is>
       </c>
       <c r="B49" s="3" t="n">
@@ -2540,31 +2540,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E49" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G49" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima, MagicStaff</t>
+          <t>MagicAnima, MagicStaff, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>LordKnight</t>
+          <t>MageKnight</t>
         </is>
       </c>
       <c r="B50" s="3" t="n">
@@ -2580,31 +2580,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G50" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MagicAnima, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>MageFighter</t>
+          <t>MasterKnight</t>
         </is>
       </c>
       <c r="B51" s="3" t="n">
@@ -2637,14 +2637,14 @@
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima, MagicStaff, MagicSword, Sword</t>
+          <t>Axe, Bow, HandAxe, Javelin, Lance, MagicAnima, MagicStaff, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>MageKnight</t>
+          <t>Paladin</t>
         </is>
       </c>
       <c r="B52" s="3" t="n">
@@ -2660,31 +2660,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E52" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F52" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G52" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima, MagicSword, Sword</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>MasterKnight</t>
+          <t>Rogue</t>
         </is>
       </c>
       <c r="B53" s="3" t="n">
@@ -2700,31 +2700,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E53" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F53" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G53" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>Axe, Bow, HandAxe, Javelin, Lance, MagicAnima, MagicStaff, MagicSword, Sword</t>
+          <t>MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>Paladin</t>
+          <t>Sage</t>
         </is>
       </c>
       <c r="B54" s="3" t="n">
@@ -2740,31 +2740,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E54" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G54" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MagicAnima, MagicStaff</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Rogue</t>
+          <t>Sniper</t>
         </is>
       </c>
       <c r="B55" s="3" t="n">
@@ -2780,31 +2780,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F55" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G55" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>MagicSword, Sword</t>
+          <t>Bow</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Sage</t>
+          <t>Swordmaster</t>
         </is>
       </c>
       <c r="B56" s="3" t="n">
@@ -2837,14 +2837,14 @@
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima, MagicStaff</t>
+          <t>MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Sniper</t>
+          <t>Warrior</t>
         </is>
       </c>
       <c r="B57" s="3" t="n">
@@ -2860,35 +2860,35 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E57" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F57" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G57" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G57" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>Bow</t>
+          <t>Axe, Bow, HandAxe</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Swordmaster</t>
+          <t>Baron</t>
         </is>
       </c>
       <c r="B58" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
@@ -2900,35 +2900,35 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E58" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F58" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G58" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>MagicSword, Sword</t>
+          <t>Axe, Bow, HandAxe, Javelin, Lance, MagicAnima, MagicStaff, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>Warrior</t>
+          <t>DarkBishop</t>
         </is>
       </c>
       <c r="B59" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
@@ -2957,14 +2957,14 @@
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>Axe, Bow, HandAxe</t>
+          <t>MagicAnima, MagicStaff</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>Baron</t>
+          <t>DarkPrince</t>
         </is>
       </c>
       <c r="B60" s="3" t="n">
@@ -2997,14 +2997,14 @@
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>Axe, Bow, HandAxe, Javelin, Lance, MagicAnima, MagicStaff, MagicSword, Sword</t>
+          <t>MagicAnima, MagicStaff</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>DarkBishop</t>
+          <t>Emperor</t>
         </is>
       </c>
       <c r="B61" s="3" t="n">
@@ -3037,14 +3037,14 @@
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima, MagicStaff</t>
+          <t>Axe, Bow, HandAxe, Javelin, Lance, MagicAnima, MagicStaff, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>DarkPrince</t>
+          <t>Queen</t>
         </is>
       </c>
       <c r="B62" s="3" t="n">
@@ -3060,9 +3060,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E62" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="F62" s="6" t="inlineStr">
@@ -3077,92 +3077,12 @@
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima, MagicStaff</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="3" t="inlineStr">
-        <is>
-          <t>Emperor</t>
-        </is>
-      </c>
-      <c r="B63" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="C63" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D63" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E63" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F63" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G63" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H63" s="3" t="inlineStr">
-        <is>
-          <t>Axe, Bow, HandAxe, Javelin, Lance, MagicAnima, MagicStaff, MagicSword, Sword</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="3" t="inlineStr">
-        <is>
-          <t>Queen</t>
-        </is>
-      </c>
-      <c r="B64" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="C64" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D64" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E64" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="F64" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G64" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H64" s="3" t="inlineStr">
-        <is>
           <t>—</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H64"/>
+  <autoFilter ref="A1:H62"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4409,17 +4329,17 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Coirpre</t>
+          <t>Laylea</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Child</t>
+          <t>Dancer</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -4432,21 +4352,21 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F34" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MagicSword, Refresh, Sword</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Laylea</t>
+          <t>Sylvia</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -4456,7 +4376,7 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -4483,12 +4403,12 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Sylvia</t>
+          <t>Sandima</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Dancer</t>
+          <t>DarkMage</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -4513,19 +4433,19 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>MagicSword, Refresh, Sword</t>
+          <t>MagicAnima</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Sandima</t>
+          <t>Deen</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>DarkMage</t>
+          <t>DragonKnight</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -4550,24 +4470,24 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima</t>
+          <t>Javelin, Lance, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Deen</t>
+          <t>Eda</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>DragonKnight</t>
+          <t>DragonRider</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -4594,17 +4514,17 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Eda</t>
+          <t>Elliot</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>DragonRider</t>
+          <t>DukeKnight</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -4617,21 +4537,21 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Javelin, Lance, MagicSword, Sword</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Elliot</t>
+          <t>Glade</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -4668,7 +4588,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Glade</t>
+          <t>Quan</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -4705,7 +4625,7 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Quan</t>
+          <t>Zain</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -4742,12 +4662,12 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Zain</t>
+          <t>DiMaggio</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>DukeKnight</t>
+          <t>Fighter</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -4765,21 +4685,21 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F43" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Axe, HandAxe</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>DiMaggio</t>
+          <t>Gerrard</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -4816,7 +4736,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Gerrard</t>
+          <t>Halvan</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -4853,7 +4773,7 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>Halvan</t>
+          <t>Johalva</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -4866,9 +4786,9 @@
           <t>M</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -4890,7 +4810,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Johalva</t>
+          <t>Osian</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -4903,9 +4823,9 @@
           <t>M</t>
         </is>
       </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -4927,12 +4847,12 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>Osian</t>
+          <t>Delmud</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Fighter</t>
+          <t>ForrestKnight</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -4950,21 +4870,21 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>Axe, HandAxe</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Delmud</t>
+          <t>Voltz</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -5001,12 +4921,12 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>Voltz</t>
+          <t>Boldor</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>ForrestKnight</t>
+          <t>General</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -5024,21 +4944,21 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F50" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Axe, Bow, HandAxe, Javelin, Lance, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>Boldor</t>
+          <t>Hannibal</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -5075,7 +4995,7 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>Hannibal</t>
+          <t>Lobos</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
@@ -5112,7 +5032,7 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>Lobos</t>
+          <t>Macbeth</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -5149,7 +5069,7 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>Macbeth</t>
+          <t>Phillip</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -5186,7 +5106,7 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Phillip</t>
+          <t>Xavier</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -5223,12 +5143,12 @@
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Xavier</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>HighPriest</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
@@ -5253,14 +5173,14 @@
       </c>
       <c r="G56" s="3" t="inlineStr">
         <is>
-          <t>Axe, Bow, HandAxe, Javelin, Lance, MagicSword, Sword</t>
+          <t>MagicAnima, MagicStaff</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Cyas</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -5273,9 +5193,9 @@
           <t>M</t>
         </is>
       </c>
-      <c r="D57" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -5297,22 +5217,22 @@
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Cyas</t>
+          <t>Deirdre</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>HighPriest</t>
+          <t>LightPriestess</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -5334,7 +5254,7 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>Deirdre</t>
+          <t>Julia</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -5371,17 +5291,17 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>Julia</t>
+          <t>Salem</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>LightPriestess</t>
+          <t>LoptoMage</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
@@ -5408,12 +5328,12 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Salem</t>
+          <t>Sigurd</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>LoptoMage</t>
+          <t>LordKnight</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
@@ -5438,19 +5358,19 @@
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima, MagicStaff</t>
+          <t>Javelin, Lance, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>Sigurd</t>
+          <t>Leif</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>LordKnight</t>
+          <t>LordLeaf</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
@@ -5475,19 +5395,19 @@
       </c>
       <c r="G62" s="3" t="inlineStr">
         <is>
-          <t>Javelin, Lance, MagicSword, Sword</t>
+          <t>MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Leif</t>
+          <t>Amid</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>LordLeaf</t>
+          <t>Mage</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
@@ -5505,21 +5425,21 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F63" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="F63" s="7" t="inlineStr">
+        <is>
+          <t>⚠️</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>MagicSword, Sword</t>
+          <t>MagicAnima, MagicStaff, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>Amid</t>
+          <t>Asbel</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -5549,14 +5469,14 @@
       </c>
       <c r="G64" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima, MagicStaff, MagicSword, Sword</t>
+          <t>MagicAnima, MagicStaff</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Asbel</t>
+          <t>Azel</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -5579,21 +5499,21 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F65" s="7" t="inlineStr">
-        <is>
-          <t>⚠️</t>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima, MagicStaff</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>Azel</t>
+          <t>Linda</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
@@ -5603,7 +5523,7 @@
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
@@ -5630,7 +5550,7 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>Linda</t>
+          <t>Miranda</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -5653,21 +5573,21 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F67" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F67" s="7" t="inlineStr">
+        <is>
+          <t>⚠️</t>
         </is>
       </c>
       <c r="G67" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MagicAnima, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>Miranda</t>
+          <t>Tailtiu</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
@@ -5677,7 +5597,7 @@
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
@@ -5697,19 +5617,19 @@
       </c>
       <c r="G68" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima, MagicSword, Sword</t>
+          <t>MagicAnima, MagicStaff, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Tailtiu</t>
+          <t>Ilios</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Mage</t>
+          <t>MageKnight</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
@@ -5727,21 +5647,21 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F69" s="7" t="inlineStr">
-        <is>
-          <t>⚠️</t>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima, MagicStaff, MagicSword, Sword</t>
+          <t>MagicAnima, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>Ilios</t>
+          <t>Olwen</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
@@ -5751,7 +5671,7 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
@@ -5778,17 +5698,17 @@
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Olwen</t>
+          <t>FakeHolyn</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>MageKnight</t>
+          <t>Mercenary</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
@@ -5808,14 +5728,14 @@
       </c>
       <c r="G71" s="3" t="inlineStr">
         <is>
-          <t>MagicAnima, MagicSword, Sword</t>
+          <t>Axe, HandAxe, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>FakeHolyn</t>
+          <t>Galzus</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
@@ -5852,7 +5772,7 @@
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>Galzus</t>
+          <t>Holyn</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
@@ -5889,7 +5809,7 @@
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>Holyn</t>
+          <t>Ralf</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
@@ -5926,12 +5846,12 @@
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Ralf</t>
+          <t>Alvar</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Mercenary</t>
+          <t>Paladin</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
@@ -5949,21 +5869,21 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F75" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="F75" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr">
         <is>
-          <t>Axe, HandAxe, MagicSword, Sword</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>Alvar</t>
+          <t>Amalda</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
@@ -5973,7 +5893,7 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
@@ -6000,7 +5920,7 @@
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Amalda</t>
+          <t>Conomor</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -6010,7 +5930,7 @@
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
@@ -6037,7 +5957,7 @@
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>Conomor</t>
+          <t>Eldigan</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
@@ -6074,7 +5994,7 @@
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Eldigan</t>
+          <t>Evan</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
@@ -6111,7 +6031,7 @@
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>Evan</t>
+          <t>Evar</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
@@ -6148,7 +6068,7 @@
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>Evar</t>
+          <t>Fred</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
@@ -6185,7 +6105,7 @@
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>Fred</t>
+          <t>Oifey</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
@@ -6198,9 +6118,9 @@
           <t>M</t>
         </is>
       </c>
-      <c r="D82" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -6222,12 +6142,12 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>Oifey</t>
+          <t>Erinys</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>Paladin</t>
+          <t>PegasusKnight</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
@@ -6235,9 +6155,9 @@
           <t>M</t>
         </is>
       </c>
-      <c r="D83" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -6245,21 +6165,21 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="F83" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="G83" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Javelin, Lance, MagicSword, Sword</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>Erinys</t>
+          <t>Femina</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -6269,12 +6189,12 @@
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="D84" s="4" t="inlineStr">
-        <is>
-          <t>✅</t>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -6296,7 +6216,7 @@
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>Femina</t>
+          <t>Misha</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
@@ -6309,9 +6229,9 @@
           <t>F</t>
         </is>
       </c>
-      <c r="D85" s="5" t="inlineStr">
-        <is>
-          <t>⬜</t>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -6333,12 +6253,12 @@
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>Misha</t>
+          <t>Karin</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>PegasusKnight</t>
+          <t>PegasusRider</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
@@ -6370,17 +6290,17 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>Karin</t>
+          <t>Coirpre</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>PegasusRider</t>
+          <t>Priest</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -6400,7 +6320,7 @@
       </c>
       <c r="G87" s="3" t="inlineStr">
         <is>
-          <t>Javelin, Lance, MagicSword, Sword</t>
+          <t>MagicStaff</t>
         </is>
       </c>
     </row>

</xml_diff>